<commit_message>
Reenfoque entero solo falta la bibliografia
</commit_message>
<xml_diff>
--- a/excels/presupuesto_proyecto.xlsx
+++ b/excels/presupuesto_proyecto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni\OCTAVO SEMESTRE\Redaccion\PropuestaProyectoDeCarrera\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2A1604-5206-40A9-95BD-F9B15DD6946F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A836E9B1-E9FF-4B91-A4DF-F6CADA578C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -140,16 +140,16 @@
     <t>Estimación base para implementación inicial.</t>
   </si>
   <si>
-    <t>96 hrs × 5 integrantes</t>
-  </si>
-  <si>
-    <t>5% aproximado</t>
-  </si>
-  <si>
-    <t>Donación académica del equipo. Tarifa de referencia Q200/hr por persona.</t>
-  </si>
-  <si>
     <t>2 años</t>
+  </si>
+  <si>
+    <t>108 hrs × 4 integrantes</t>
+  </si>
+  <si>
+    <t>Donación académica del equipo. Tarifa de referencia Q100/hr por persona.</t>
+  </si>
+  <si>
+    <t>15% aproximado</t>
   </si>
 </sst>
 </file>
@@ -667,7 +667,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C5" s="10">
         <v>240</v>
@@ -793,11 +793,11 @@
         <v>28</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C14" s="11">
-        <f>96*5*100</f>
-        <v>48000</v>
+        <f>108*4*100</f>
+        <v>43200</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>36</v>
@@ -810,7 +810,7 @@
       <c r="B15" s="18"/>
       <c r="C15" s="12">
         <f>SUM(C5:C14)</f>
-        <v>49990</v>
+        <v>45190</v>
       </c>
       <c r="D15" s="6"/>
     </row>
@@ -819,7 +819,7 @@
         <v>30</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C16" s="13">
         <f>SUM(C5:C13)*0.15</f>
@@ -836,7 +836,7 @@
       <c r="B17" s="19"/>
       <c r="C17" s="14">
         <f>C15+C16</f>
-        <v>50288.5</v>
+        <v>45488.5</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>33</v>

</xml_diff>